<commit_message>
Publish season run run-2026-10-31T09-20
</commit_message>
<xml_diff>
--- a/latest/season_plan_spond_games.xlsx
+++ b/latest/season_plan_spond_games.xlsx
@@ -2091,7 +2091,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 14:30 • Slutt: 16:20</t>
+          <t>Start: 13:30 • Slutt: 15:50</t>
         </is>
       </c>
     </row>
@@ -3204,7 +3204,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 10:30 • Slutt: 12:50</t>
+          <t>Start: 10:30 • Slutt: 13:00</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4155,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 13:00 • Slutt: 14:50</t>
+          <t>Start: 13:00 • Slutt: 15:20</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 17:00 • Slutt: 18:50</t>
+          <t>Start: 16:30 • Slutt: 18:50</t>
         </is>
       </c>
     </row>
@@ -5447,7 +5447,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 15:00 • Slutt: 17:19</t>
+          <t>Start: 15:00 • Slutt: 17:20</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6114,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 12:00 • Slutt: 13:50</t>
+          <t>Start: 12:00 • Slutt: 14:20</t>
         </is>
       </c>
     </row>
@@ -6455,7 +6455,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 12:30 • Slutt: 14:09</t>
+          <t>Start: 12:30 • Slutt: 14:10</t>
         </is>
       </c>
     </row>
@@ -7154,7 +7154,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 14:15 • Slutt: 16:49</t>
+          <t>Start: 14:15 • Slutt: 16:50</t>
         </is>
       </c>
     </row>
@@ -9845,7 +9845,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 14:30 • Slutt: 16:20</t>
+          <t>Start: 14:30 • Slutt: 16:50</t>
         </is>
       </c>
     </row>
@@ -10868,7 +10868,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 13:30 • Slutt: 15:09</t>
+          <t>Start: 13:30 • Slutt: 15:10</t>
         </is>
       </c>
     </row>
@@ -11908,7 +11908,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 13:30 • Slutt: 15:20</t>
+          <t>Start: 13:00 • Slutt: 14:50</t>
         </is>
       </c>
     </row>
@@ -12518,7 +12518,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 15:30 • Slutt: 17:20</t>
+          <t>Start: 15:00 • Slutt: 17:20</t>
         </is>
       </c>
     </row>
@@ -12859,7 +12859,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 14:15 • Slutt: 16:34</t>
+          <t>Start: 14:15 • Slutt: 16:35</t>
         </is>
       </c>
     </row>
@@ -13950,9 +13950,9 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -13973,7 +13973,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Deltakende lag: Frisk Asker, Jar, Jutul Kittens, Skien</t>
+          <t>Deltakende lag: Frisk Asker, Wildcats Turkis, Wildcats Rosa, Skien</t>
         </is>
       </c>
     </row>
@@ -14017,7 +14017,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -14030,7 +14030,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -14066,12 +14066,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -14089,7 +14089,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -14102,7 +14102,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -16743,7 +16743,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 14:30 • Slutt: 16:20</t>
+          <t>Start: 14:30 • Slutt: 16:50</t>
         </is>
       </c>
     </row>
@@ -19059,7 +19059,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 13:00 • Slutt: 15:35</t>
+          <t>Start: 13:00 • Slutt: 16:00</t>
         </is>
       </c>
     </row>
@@ -21392,7 +21392,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 10:30 • Slutt: 12:50</t>
+          <t>Start: 10:30 • Slutt: 13:00</t>
         </is>
       </c>
     </row>
@@ -22684,7 +22684,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 17:30 • Slutt: 19:50</t>
+          <t>Start: 17:30 • Slutt: 20:00</t>
         </is>
       </c>
     </row>
@@ -24481,7 +24481,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 12:00 • Slutt: 13:50</t>
+          <t>Start: 12:00 • Slutt: 14:20</t>
         </is>
       </c>
     </row>
@@ -25611,7 +25611,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 15:00 • Slutt: 16:50</t>
+          <t>Start: 15:30 • Slutt: 17:50</t>
         </is>
       </c>
     </row>
@@ -27393,9 +27393,9 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -27416,14 +27416,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Deltakende lag: Frisk Asker, Jar, Jutul Kittens, Skien</t>
+          <t>Deltakende lag: Frisk Asker, Wildcats Turkis, Wildcats Rosa, Skien</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 13:00 • Slutt: 15:00</t>
+          <t>Start: 13:00 • Slutt: 14:20</t>
         </is>
       </c>
     </row>
@@ -27460,7 +27460,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -27473,7 +27473,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -27509,12 +27509,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -27532,7 +27532,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -27545,7 +27545,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -27602,7 +27602,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 15:00 • Slutt: 16:50</t>
+          <t>Start: 14:30 • Slutt: 16:50</t>
         </is>
       </c>
     </row>
@@ -30172,9 +30172,9 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -30195,7 +30195,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Deltakende lag: Frisk Asker, Jar, Jutul Kittens, Skien</t>
+          <t>Deltakende lag: Frisk Asker, Wildcats Turkis, Wildcats Rosa, Skien</t>
         </is>
       </c>
     </row>
@@ -30239,7 +30239,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -30252,7 +30252,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -30288,12 +30288,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -30311,7 +30311,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -30324,7 +30324,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -30739,7 +30739,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 12:00 • Slutt: 13:50</t>
+          <t>Start: 12:00 • Slutt: 14:20</t>
         </is>
       </c>
     </row>
@@ -31080,7 +31080,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 16:30 • Slutt: 18:50</t>
+          <t>Start: 16:30 • Slutt: 19:00</t>
         </is>
       </c>
     </row>
@@ -33323,7 +33323,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 12:00 • Slutt: 14:20</t>
+          <t>Start: 12:00 • Slutt: 14:30</t>
         </is>
       </c>
     </row>
@@ -34005,7 +34005,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 15:00 • Slutt: 17:20</t>
+          <t>Start: 15:00 • Slutt: 17:30</t>
         </is>
       </c>
     </row>
@@ -35062,7 +35062,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 15:00 • Slutt: 16:40</t>
+          <t>Start: 15:00 • Slutt: 17:00</t>
         </is>
       </c>
     </row>
@@ -35241,7 +35241,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 15:00 • Slutt: 17:20</t>
+          <t>Start: 15:00 • Slutt: 17:30</t>
         </is>
       </c>
     </row>
@@ -35553,8 +35553,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -35575,7 +35575,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Deltakende lag: Frisk Asker, Jar, Jutul Kittens, Ringerike 1, Skien</t>
+          <t>Deltakende lag: Frisk Asker, Wildcats Turkis, Wildcats Rosa, Ringerike 1, Skien</t>
         </is>
       </c>
     </row>
@@ -35614,7 +35614,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -35632,7 +35632,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -35668,7 +35668,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -35727,7 +35727,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -35740,7 +35740,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -35776,12 +35776,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -35814,7 +35814,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
     </row>
@@ -35829,7 +35829,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
     </row>
@@ -37379,7 +37379,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 15:30 • Slutt: 17:20</t>
+          <t>Start: 15:00 • Slutt: 17:20</t>
         </is>
       </c>
     </row>
@@ -39867,7 +39867,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 12:00 • Slutt: 13:50</t>
+          <t>Start: 12:00 • Slutt: 14:20</t>
         </is>
       </c>
     </row>
@@ -41338,7 +41338,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 15:00 • Slutt: 16:50</t>
+          <t>Start: 14:30 • Slutt: 16:50</t>
         </is>
       </c>
     </row>
@@ -41858,7 +41858,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 12:00 • Slutt: 14:20</t>
+          <t>Start: 12:00 • Slutt: 14:30</t>
         </is>
       </c>
     </row>
@@ -42169,9 +42169,9 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -42192,7 +42192,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Deltakende lag: Frisk Asker, Jar, Jutul Kittens, Skien</t>
+          <t>Deltakende lag: Frisk Asker, Wildcats Turkis, Wildcats Rosa, Skien</t>
         </is>
       </c>
     </row>
@@ -42236,7 +42236,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -42249,7 +42249,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -42285,12 +42285,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -42308,7 +42308,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -42321,7 +42321,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -43346,7 +43346,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 15:00 • Slutt: 16:50</t>
+          <t>Start: 14:00 • Slutt: 16:20</t>
         </is>
       </c>
     </row>
@@ -43687,7 +43687,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 12:30 • Slutt: 14:10</t>
+          <t>Start: 12:30 • Slutt: 14:20</t>
         </is>
       </c>
     </row>
@@ -43866,7 +43866,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 12:00 • Slutt: 14:20</t>
+          <t>Start: 12:00 • Slutt: 14:30</t>
         </is>
       </c>
     </row>
@@ -48248,7 +48248,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 16:00 • Slutt: 18:36</t>
+          <t>Start: 16:00 • Slutt: 18:35</t>
         </is>
       </c>
     </row>
@@ -51190,7 +51190,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 12:00 • Slutt: 13:50</t>
+          <t>Start: 12:00 • Slutt: 14:20</t>
         </is>
       </c>
     </row>
@@ -54371,9 +54371,9 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -54394,7 +54394,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Deltakende lag: Frisk Asker, Jar, Jutul Kittens, Skien</t>
+          <t>Deltakende lag: Frisk Asker, Wildcats Turkis, Wildcats Rosa, Skien</t>
         </is>
       </c>
     </row>
@@ -54438,7 +54438,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -54451,7 +54451,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -54487,12 +54487,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -54510,7 +54510,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -54523,7 +54523,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -54759,7 +54759,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 15:00 • Slutt: 17:34</t>
+          <t>Start: 15:00 • Slutt: 17:35</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish season run run-2026-11-01T08-56
</commit_message>
<xml_diff>
--- a/latest/season_plan_spond_games.xlsx
+++ b/latest/season_plan_spond_games.xlsx
@@ -23850,7 +23850,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>(AVLYST) 06.03.2027 (lørdag) — U12 — Baerum ishall</t>
+          <t>06.03.2027 (lørdag) — U12 — Baerum ishall</t>
         </is>
       </c>
     </row>
@@ -23871,7 +23871,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 14:20 • Slutt: 16:00</t>
+          <t>Start: 18:15 • Slutt: 19:55</t>
         </is>
       </c>
     </row>
@@ -33643,7 +33643,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>(AVLYST) 14.11.2026 (lørdag) — U11 — Baerum ishall</t>
+          <t>14.11.2026 (lørdag) — U11 — Baerum ishall</t>
         </is>
       </c>
     </row>
@@ -36407,7 +36407,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>(AVLYST) 21.11.2026 (lørdag) — U9 — Baerum ishall</t>
+          <t>21.11.2026 (lørdag) — U9 — Baerum ishall</t>
         </is>
       </c>
     </row>
@@ -36428,7 +36428,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Start: 17:20 • Slutt: 19:55</t>
+          <t>Start: 17:30 • Slutt: 20:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish season run run-2026-11-01T09-49
</commit_message>
<xml_diff>
--- a/latest/season_plan_spond_games.xlsx
+++ b/latest/season_plan_spond_games.xlsx
@@ -23850,7 +23850,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>06.03.2027 (lørdag) — U12 — Baerum ishall</t>
+          <t>(AVLYST) 06.03.2027 (lørdag) — U12 — Baerum ishall</t>
         </is>
       </c>
     </row>
@@ -33643,7 +33643,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>14.11.2026 (lørdag) — U11 — Baerum ishall</t>
+          <t>(AVLYST) 14.11.2026 (lørdag) — U11 — Baerum ishall</t>
         </is>
       </c>
     </row>
@@ -36407,7 +36407,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>21.11.2026 (lørdag) — U9 — Baerum ishall</t>
+          <t>(AVLYST) 21.11.2026 (lørdag) — U9 — Baerum ishall</t>
         </is>
       </c>
     </row>

</xml_diff>